<commit_message>
Template fully editable/unlocked; header title on one line
Parity with v3: template sheet protection removed (all cells editable,
non-blocking drop-downs), download link cache-busted (?v=2); header <h1>
0.8rem + nowrap for a single-line title. Bump style.css (?v=20260707d).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IDB_New_Pole_Installation_Template.xlsx
+++ b/IDB_New_Pole_Installation_Template.xlsx
@@ -8022,7 +8022,6 @@
       <c r="X258" s="23" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="CE4B"/>
   <mergeCells count="12">
     <mergeCell ref="A3:X3"/>
     <mergeCell ref="J4:K4"/>
@@ -8038,35 +8037,35 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <dataValidations count="10">
-    <dataValidation sqref="B8:B258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Business Unit" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="B8:B258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Business Unit" prompt="Pick from the list, or type your own." type="list">
       <formula1>'Lists'!$A$2:$A$2</formula1>
     </dataValidation>
-    <dataValidation sqref="C8:C258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Undertaking" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="C8:C258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Undertaking" prompt="Pick from the list, or type your own." type="list">
       <formula1>'Lists'!$B$2:$B$11</formula1>
     </dataValidation>
-    <dataValidation sqref="D8:D258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Feeder" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="D8:D258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Feeder" prompt="Pick from the list, or type your own." type="list">
       <formula1>'Lists'!$C$2:$C$57</formula1>
     </dataValidation>
-    <dataValidation sqref="E8:E258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="DT Name" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="E8:E258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="DT Name" prompt="Pick from the list, or type your own." type="list">
       <formula1>'Lists'!$D$2:$D$986</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Pole Category" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="H8:H258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Pole Category" prompt="Pick from the list, or type your own." type="list">
       <formula1>"New Install"</formula1>
     </dataValidation>
-    <dataValidation sqref="I8:I258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Type of Pole" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="I8:I258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Type of Pole" prompt="Pick from the list, or type your own." type="list">
       <formula1>'Lists'!$E$2:$E$5</formula1>
     </dataValidation>
-    <dataValidation sqref="K8:K258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Reason for Installation" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="K8:K258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Reason for Installation" prompt="Pick from the list, or type your own." type="list">
       <formula1>"New Extension,Replacement of Bad Pole,Network Expansion,Reinforcement,Road Expansion / Relocation"</formula1>
     </dataValidation>
-    <dataValidation sqref="X8:X258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Status" prompt="Select from the drop-down." type="list">
+    <dataValidation sqref="X8:X258" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Pick from the list, or type your own." type="list">
       <formula1>"Pending GIS Capture,Captured — Complete"</formula1>
     </dataValidation>
-    <dataValidation sqref="M9:M258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid coordinate" error="Enter decimal degrees (e.g. 6.5362)." type="decimal" operator="between">
+    <dataValidation sqref="M9:M258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
       <formula1>-90</formula1>
       <formula2>180</formula2>
     </dataValidation>
-    <dataValidation sqref="N9:N258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid coordinate" error="Enter decimal degrees (e.g. 6.5362)." type="decimal" operator="between">
+    <dataValidation sqref="N9:N258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
       <formula1>-90</formula1>
       <formula2>180</formula2>
     </dataValidation>

</xml_diff>